<commit_message>
Add exit month metadata to respondent intake
</commit_message>
<xml_diff>
--- a/frontend/public/templates/verisight-respondenten-template.xlsx
+++ b/frontend/public/templates/verisight-respondenten-template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,26 +28,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001E3A8A"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -55,31 +46,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D1D5DB"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D1D5DB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D1D5DB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D1D5DB"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,13 +418,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,76 +446,88 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>exit_month</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>annual_salary_eur</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>anne@bedrijf.nl</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>62000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>karim@bedrijf.nl</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Customer Service</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>uitvoerend</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sanne@bedrijf.nl</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>specialist</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>52000</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>karim@bedrijf.nl</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>manager</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>64000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>sanne@bedrijf.nl</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>senior</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>58000</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>42000</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"uitvoerend,specialist,senior,manager,director,c_level"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -555,83 +541,81 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Gebruik</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Gebruik ??n respondent per rij. Laat de kolomnamen in rij 1 ongewijzigd.</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Aanleverinstructie Verisight respondentenbestand</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Verplicht</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>email</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Verplichte kolom</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sterk aanbevolen</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>department, role_level</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>Voor retrospectieve batches aanbevolen</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verplicht voor uitnodigingen per e-mail.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Optionele kolommen</t>
+          <t>exit_month (formaat YYYY-MM, bijvoorbeeld 2026-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Optioneel</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>annual_salary_eur</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>department</t>
+          <t>Toegestane role_level-waarden</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bijv. Operations, Sales, HR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>role_level</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Een van: uitvoerend, specialist, senior, manager, director, c_level.</t>
+          <t>uitvoerend, specialist, senior, manager, director, c_level</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>annual_salary_eur</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Alleen cijfers, zonder euroteken.</t>
+          <t>Gebruik exit_month vooral bij een Baseline / retrospectieve ExitScan, zodat recency in rapportage en methodiek duidelijker geduid kan worden.</t>
         </is>
       </c>
     </row>

</xml_diff>